<commit_message>
Update reports 2026-06-15 10:37
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-06-15.xlsx
+++ b/gex_pivot_levels_2026-06-15.xlsx
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$645.42K</t>
+          <t>-$602.39K</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$10.40M</t>
+          <t>+$9.71M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>+$30.92M</t>
+          <t>+$32.26M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$46.16M</t>
+          <t>+$48.17M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>+$3.27M</t>
+          <t>+$3.49M</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>+$4.64M</t>
+          <t>+$4.94M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>+$19.60M</t>
+          <t>+$20.84M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$29.00M</t>
+          <t>+$30.83M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>+$4.11M</t>
+          <t>+$4.38M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$5.81M</t>
+          <t>+$6.19M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -4001,12 +4001,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>+$30.92M</t>
+          <t>+$32.26M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$46.16M</t>
+          <t>+$48.17M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -4039,12 +4039,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$19.60M</t>
+          <t>+$20.84M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$29.00M</t>
+          <t>+$30.83M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -4597,12 +4597,12 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>-$645.42K</t>
+          <t>-$602.39K</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$10.40M</t>
+          <t>+$9.71M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -4763,146 +4763,146 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>30017.79</v>
+        <v>7538.54</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>730</v>
+        <v>7535</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>+$3.33M</t>
+          <t>+$4.38M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>+$6.12M</t>
+          <t>+$6.19M</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>30017.79</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>730</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>+$3.33M</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>+$6.12M</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>7538.54</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>7535</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="B27" s="5" t="n">
+        <v>7518.54</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>7515</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$4.11M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$5.81M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>+$3.49M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$4.94M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B28" s="2" t="n">
         <v>4424.09</v>
       </c>
-      <c r="C27" s="2" t="n">
+      <c r="C28" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>+$3.49M</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>+$4.88M</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>7357.35</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>734</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>+$2.00M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$4.84M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4911,36 +4911,40 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>4740.1</v>
+        <v>7357.35</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>90</v>
+        <v>734</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>-$331.54K</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>+$2.00M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$4.73M</t>
+          <t>+$4.84M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -4949,24 +4953,24 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>4266.09</v>
+        <v>4740.1</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>+$2.63M</t>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-$331.54K</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>+$4.70M</t>
+          <t>+$4.73M</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -4979,40 +4983,36 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7518.54</v>
+        <v>4266.09</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>7515</v>
+        <v>81</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>+$3.27M</t>
+          <t>+$2.63M</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>+$4.64M</t>
+          <t>+$4.70M</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">

</xml_diff>